<commit_message>
feat: adding failed-focus question feature
</commit_message>
<xml_diff>
--- a/raw_csv_quiz/Quiz_Week01.xlsx
+++ b/raw_csv_quiz/Quiz_Week01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LearningHub\ai-2y-journey\06-other\flashcard-app\raw_csv_quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50EDA334-91C2-4C2F-B09C-A452F905C79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6CF83C-71FA-4D32-98A3-14E9B0F82340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="1346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="1366">
   <si>
     <t>Question</t>
   </si>
@@ -3982,10 +3982,6 @@
     <t>Edge locations are AWS sites positioned close to users to reduce latency.</t>
   </si>
   <si>
-    <t>"1.An ecommerce company has migrated its IT infrastructure from an on-premises data center to the AWS Cloud.
-Which cost is the company’s direct responsibility?</t>
-  </si>
-  <si>
     <t>Cost of application software licenses</t>
   </si>
   <si>
@@ -4124,6 +4120,142 @@
   </si>
   <si>
     <t>When move on on-premises</t>
+  </si>
+  <si>
+    <t>When you build your own data center (on-premises), you buy the servers, you plug them into the wall, and you lock the doors. You own the hardware. The main benefit of doing this is that you have 100% physical control. Some companies have to do this because of very strict government regulations, security compliance rules, or because they need highly customized hardware that AWS doesn't offer.</t>
+  </si>
+  <si>
+    <t>1. Cloud-Native (All-in Cloud): You don't guess capacity (Auto-scaling), you trade capital expense for variable expense (pay-as-you-go), and you stop maintaining physical hardware.
+2. On-Premises (Private Cloud): You have total physical control, high upfront costs (CapEx), and you are 100% responsible for hardware maintenance and physical security.
+3. Hybrid: A mix of both. Usually used when a company wants to use the cloud but has to keep some data on-premises due to strict laws, compliance, or legacy systems that can't move to the cloud yet.</t>
+  </si>
+  <si>
+    <t>In AWS terminology, Agility specifically means Speed.
+Before the cloud, if a developer wanted to test a new app, they had to ask the IT team to order a physical server. It took weeks to order, ship, install, and configure.
+In the AWS Cloud, you can provision (turn on) and deprovision (turn off) thousands of servers in minutes. This allows companies to experiment faster and innovate quicker. That speed and flexibility is exactly what AWS calls "Agility."</t>
+  </si>
+  <si>
+    <t>"Six Advantages of Cloud Computing." AWS loves to test these exactly as they are written below. I will give you the cheat sheet for matching the AWS Advantage to its exam definition:
+1. Increase speed and agility: Spin up resources in minutes (provision/deprovision quickly).
+2. Trade capital expense for variable expense: Pay-as-you-go. No huge upfront costs.
+3. Stop guessing capacity: Use Auto Scaling to match traffic perfectly.
+4. Benefit from massive economies of scale: Because AWS is so huge, they get cheaper hardware and pass the savings to you (lower pay-as-you-go prices).
+5. Stop spending money running and maintaining data centers: Focus on your own customers, let AWS manage the heavy lifting of the physical servers.
+6. Go global in minutes: Deploy your app in different Regions around the world with a few clicks.</t>
+  </si>
+  <si>
+    <t>1. Scope (Single Country) + Cost/Simple: Because the customers are in one country, a Single-Region is perfect. Going Multi-Region is very expensive and very complicated (which would make the CFO mad).
+2. Performance (&lt;10ms latency): In AWS, Availability Zones (AZs) inside the same Region are physically located tens of miles apart and connected by dedicated, super-fast fiber optic cables. AWS literally guarantees single-digit millisecond latency between AZs.
+3. Availability (Immediate failover): This is where Active/Active and Synchronous Replication come in. Because both AZs are actively taking traffic at the same time, if one data center completely loses power, the other one is already running. The customer won't even notice the failure.</t>
+  </si>
+  <si>
+    <t>1. Active/Active vs. Active/Passive (Standby)
+Active/Active: Think of a supermarket with two cashiers working at the same time. Both are taking customers. If Cashier A faints, Cashier B just keeps working. There is zero downtime. It is the most highly available, but it costs more because both servers are running at full power all the time.
+Active/Passive (also called Multi-AZ with Standby): Think of a supermarket with one cashier working (Active), and one employee sweeping the floor nearby (Passive/Standby). If the cashier faints, the sweeper drops the broom, walks over, logs into the register, and starts taking customers. There is a brief pause (failover time). It's cheaper, but there is a slight delay.
+2. Synchronous vs. Asynchronous Replication (Copying Data)
+Synchronous (Same time): When a customer buys a shirt, the database writes the receipt to Server A and Server B at the exact same time. It waits until both confirm before telling the customer "Success!" Zero data loss.
+Asynchronous (Catch-up later): The database writes the receipt to Server A, tells the customer "Success!", and then copies the receipt to Server B in the background a few seconds later. If Server A explodes before it copies, data is lost.
+-&gt; Summary for the Exam:
+If a question demands zero downtime, zero data loss, or immediate failover, you always look for Multi-AZ, Active/Active, and Synchronous.</t>
+  </si>
+  <si>
+    <t>Loose Coupling means building your application out of separate, independent pieces that talk to each other, but don't rely on each other to survive.
+Imagine you buy a separate TV and a separate DVD player, and connect them with a cable. If the DVD player catches on fire, does the TV break? No! The TV still works perfectly fine; you just can't watch DVDs right now. You can easily unplug the broken DVD player, throw it away, and plug in a new one.
+In AWS, if your Web Server and your Database are "loosely coupled," and the Database crashes, the Web Server won't crash. It will just politely tell the user, "Hey, we received your order and will process it shortly," while waiting for the Database to come back online.</t>
+  </si>
+  <si>
+    <t>AWS heavily tests the concept of decoupling. Here are the magic buzzwords and services you need to memorize:
+1. The Magic Phrase:
+If a question asks how to "reduce interdependencies," "prevent single points of failure," or "make components independent," the answer is always Loose Coupling (or Decoupling).
+2. Microservices:
+When a company takes a giant "Monolithic" app and breaks it into tiny, loosely coupled pieces, those pieces are called Microservices. (Example: The Amazon website has a separate microservice for the "Add to Cart" button, a separate one for the "Reviews," and a separate one for "Recommended Items").
+3. Amazon SQS (Simple Queue Service):
+If the exam asks which AWS service helps you achieve loose coupling, the number one answer is Amazon SQS. It acts as a waiting room (a queue) between two parts of an application. If the receiving server crashes, the messages just sit safely in the SQS queue until a new server spins up to read them. No data is lost, and nothing crashes!</t>
+  </si>
+  <si>
+    <t>This question isn't about legal compliance; it's a Disaster Recovery question. In the AWS world, "high political instability" is treated exactly like a massive hurricane or an earthquake—it represents a high risk that the entire country's power grid or internet might be shut down.
+An AWS Region is a physical geographic area in the world (like Tokyo, Ireland, or Northern Virginia). If a company is in an area where the entire country's internet or power could go down due to political unrest, the only way to ensure the application stays alive (business continuity) is to have a copy of the application running in a completely different, stable part of the world. If Region A goes completely dark, Region B instantly takes over.</t>
+  </si>
+  <si>
+    <t>1. Fault Tolerance / High Availability = Multi-AZ
+The Disaster: A hard drive fails, a rack catches fire, or a localized flood hits a single data center.
+The Solution: Multi-AZ. Because AZs are miles apart, one AZ dying won't kill the other. It protects against local disasters.
+2. Disaster Recovery / Business Continuity = Multi-Region
+The Disaster: A massive earthquake, a nuclear event, or extreme political instability wipes out an entire geographic area's infrastructure.
+The Solution: Multi-Region. Because Regions are completely independent and scattered globally, an event that destroys one Region won't affect the others. It protects against regional/country-wide disasters.
+3. The Compliance Trap (Data Sovereignty)
+If the exam question had said: "A company's local government passed a strict law stating citizen data cannot leave the country's borders," THEN your logic would be 100% correct! You would have to keep the data local. But whenever you see "resilience" or "disaster recovery," think Multi-Region.</t>
+  </si>
+  <si>
+    <t>B. Multi-Region deployment is used only for global applications and is not relevant to disaster recovery planning.
+This statement is a massive lie. As we just learned in the last question, Multi-Region is the ultimate Disaster Recovery (DR) strategy! If a whole Region gets wiped out by a disaster, you failover to the second Region. Therefore, saying it is "not relevant to disaster recovery" is completely false. Since it's false, it's the correct answer to the question.</t>
+  </si>
+  <si>
+    <t>Imagine your company's database crashes at 12:00 PM (Noon).
+1. RTO (Recovery TIME Objective): "How long can we stay offline?"
+This is about Downtime.
+If your boss says, "We need the system back online by 2:00 PM," your RTO is 2 hours.
+Trick to remember: RTO = Time until the system is fixed.
+2. RPO (Recovery POINT Objective): "How much data can we afford to lose?"
+This is about Data Loss (Backups).
+If your last backup was taken at 10:00 AM, and the crash happened at 12:00 PM, you just lost 2 hours of customer data. If your boss says, "It is unacceptable to lose more than 1 hour of data," your RPO is 1 hour (meaning you better be taking backups every single hour!).
+Trick to remember: RPO = Past data. What Point in the past are we restoring from?
+1. Read carefully: AWS loves to throw "Which is NOT true" or "Which is INCORRECT" questions at you. Take a deep breath and read the prompt twice!
+2. Absolutes are usually lies: In AWS exam questions, if an option uses a word like "ONLY," "ALWAYS," or "NEVER," be very suspicious. (Notice how option B said Multi-Region is used only for global apps? That was a huge hint that it was the false statement!).
+3. RPO vs RTO Cheat Sheet:
+RTO: Downtime. How fast do we need to recover?
+RPO: Data loss. How frequently do we need to take backups?</t>
+  </si>
+  <si>
+    <t>B. Data is not replicated outside of a region unless you configure it.
+Here is the exact reason why B is the right answer, and why C is a trap.
+Why the answer is B (The True Statement):
+This question is testing a massive, foundational rule of AWS called Data Sovereignty.
+Many countries have extremely strict laws about where citizen data can live. For example, if you are a hospital in Germany, by law, your patient data must stay inside Germany.
+Because of these laws, AWS makes a strict promise: AWS will NEVER move your data out of the Region you selected unless you explicitly click a button and tell them to. If you put data in the Frankfurt (Germany) Region, it stays in Frankfurt forever. It will never automatically copy to the US or Japan. You have to manually set up Cross-Region Replication if you want it to move.</t>
+  </si>
+  <si>
+    <t>1. The Golden Rule of Data Location:
+You own your data. AWS acts as the landlord. The landlord will never pack up your apartment and move your stuff to a different city without your permission. Data never leaves a Region automatically.
+2. Regional Services vs. AZ-Specific Services:
+The exam will test you on which services exist across a whole Region, and which are stuck in just one Availability Zone. Memorize these two heavily tested examples:
+2.1. Amazon S3 (Simple Storage Service): It is a Regional service. It automatically copies your data to multiple AZs in the background. Highly available by default.
+2.2. Amazon EBS (Elastic Block Store): It is an AZ-specific service. It lives in ONE Availability Zone. If you want a copy in another AZ, you have to manually take a Snapshot (backup) of it.</t>
+  </si>
+  <si>
+    <t>AWS IAM is the service where you create usernames, passwords, and permissions for your team.
+Think about it like a Passport. If you hire a new developer named Sarah, you don't want her to only exist in the "US-East (Virginia)" Region. If she needs to go fix a server in "EU-West (Ireland)", you want her same login to work there too. Because identities and permissions need to apply to your entire AWS account no matter where you are building things, IAM is a Global service.</t>
+  </si>
+  <si>
+    <t>The "Big 4" Global Services to Memorize:
+1. AWS IAM (Identity and Access Management): Users, groups, and passwords.
+2. Amazon Route 53: This is AWS's DNS service (it routes web traffic like an internet phonebook). The internet is global, so Route 53 is global.
+3. Amazon CloudFront: This is a Content Delivery Network (CDN). It uses Edge Locations all around the world to deliver images and videos fast.
+4. AWS WAF (Web Application Firewall) &amp; Shield: Since CloudFront and Route 53 are on the edge of the global internet, the security protecting them from hackers (DDoS attacks) also has to be global.</t>
+  </si>
+  <si>
+    <t>AWS Availability Zones (AZs) are usually located a few miles apart (no more than 60 miles). To make sure your application doesn't freeze when saving data, AWS connects these buildings with their own private, dedicated, super-fast fiber-optic cables. Because they are relatively close and connected by fiber, the data travels at the speed of light (under 1 millisecond). This ultra-fast connection is the only physical way Synchronous Replication is possible!</t>
+  </si>
+  <si>
+    <t>You will definitely get questions about how AWS physical infrastructure is built. Memorize these facts about Availability Zones (AZs):
+1. What is an AZ? It is one or more physical data centers.
+2. Independence: Every AZ has its own separate and independent power supply, cooling, and network connectivity.
+3. Distance: AZs inside a Region are miles apart (to protect against local disasters like floods) but close enough to have single-digit millisecond latency (fast enough for real-time data copying).
+4. Network: They are connected via redundant, private, high-speed fiber-optic networking.
+Exam Cheat Code for Replication:
+1. If a question asks about copying data within a Region (Multi-AZ) = It is Synchronous (Real-time/Fast).
+2. If a question asks about copying data across the globe (Multi-Region) = It is Asynchronous (Slight delay/Catch up later).</t>
+  </si>
+  <si>
+    <t>An ecommerce company has migrated its IT infrastructure from an on-premises data center to the AWS Cloud.
+Which cost is the company’s direct responsibility?</t>
+  </si>
+  <si>
+    <t>When you move to AWS, you are renting virtual space. If you decide to install a piece of software on your rented server (like a paid ecommerce platform, a special database, or even a specific version of Windows), you have to bring the license for it, or pay for it. AWS just provides the "empty" virtual server; what you put inside it (your data, your apps, your software licenses) is 100% your responsibility.</t>
+  </si>
+  <si>
+    <t>1. AWS is responsible for security OF the Cloud: Think Physical. AWS is responsible for the physical buildings, physical servers, physical network cables, the power, the cooling, and the hypervisor (the software that splits physical servers into virtual ones).
+2. The Customer is responsible for security IN the Cloud: Think Digital. You are responsible for everything you put inside the cloud. Your customer data, your passwords (IAM), your software, your application licenses, and your virtual firewall rules.</t>
   </si>
 </sst>
 </file>
@@ -4164,9 +4296,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4498,10 +4633,10 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
@@ -4524,10 +4659,10 @@
         <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="H2" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -4550,7 +4685,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -4568,6 +4703,12 @@
       </c>
       <c r="F4" t="s">
         <v>23</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>1347</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>1348</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -6410,7 +6551,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>421</v>
       </c>
@@ -6429,8 +6570,14 @@
       <c r="F97" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G97" s="2" t="s">
+        <v>1359</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>1360</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>422</v>
       </c>
@@ -6450,7 +6597,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>426</v>
       </c>
@@ -6470,8 +6617,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" t="s">
+    <row r="100" spans="1:8" ht="331.2" x14ac:dyDescent="0.3">
+      <c r="A100" s="2" t="s">
         <v>431</v>
       </c>
       <c r="B100" t="s">
@@ -6489,8 +6636,14 @@
       <c r="F100" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G100" t="s">
+        <v>1345</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>1346</v>
+      </c>
+    </row>
+    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>436</v>
       </c>
@@ -6510,7 +6663,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>441</v>
       </c>
@@ -6530,7 +6683,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>446</v>
       </c>
@@ -6550,7 +6703,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>451</v>
       </c>
@@ -6570,7 +6723,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>456</v>
       </c>
@@ -6590,7 +6743,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>461</v>
       </c>
@@ -6610,7 +6763,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>466</v>
       </c>
@@ -6630,7 +6783,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>471</v>
       </c>
@@ -6650,7 +6803,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>476</v>
       </c>
@@ -6670,7 +6823,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>481</v>
       </c>
@@ -6690,7 +6843,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>486</v>
       </c>
@@ -6710,7 +6863,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>487</v>
       </c>
@@ -7050,7 +7203,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>553</v>
       </c>
@@ -7070,7 +7223,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>556</v>
       </c>
@@ -7090,7 +7243,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>561</v>
       </c>
@@ -7110,8 +7263,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" t="s">
+    <row r="132" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A132" s="2" t="s">
         <v>566</v>
       </c>
       <c r="B132" t="s">
@@ -7129,8 +7282,14 @@
       <c r="F132" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G132" s="2" t="s">
+        <v>1349</v>
+      </c>
+      <c r="H132" s="2" t="s">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="133" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>571</v>
       </c>
@@ -7150,7 +7309,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>576</v>
       </c>
@@ -7170,7 +7329,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>581</v>
       </c>
@@ -7190,7 +7349,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>586</v>
       </c>
@@ -7210,7 +7369,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>591</v>
       </c>
@@ -7230,7 +7389,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>596</v>
       </c>
@@ -7250,7 +7409,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>601</v>
       </c>
@@ -7270,7 +7429,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>603</v>
       </c>
@@ -7290,7 +7449,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>605</v>
       </c>
@@ -7310,7 +7469,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>610</v>
       </c>
@@ -7330,7 +7489,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>613</v>
       </c>
@@ -7350,7 +7509,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>614</v>
       </c>
@@ -7690,7 +7849,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>678</v>
       </c>
@@ -7710,7 +7869,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>682</v>
       </c>
@@ -7730,7 +7889,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>683</v>
       </c>
@@ -7750,7 +7909,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>685</v>
       </c>
@@ -7770,7 +7929,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>690</v>
       </c>
@@ -7789,8 +7948,14 @@
       <c r="F165" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G165" s="2" t="s">
+        <v>1357</v>
+      </c>
+      <c r="H165" s="2" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="166" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>695</v>
       </c>
@@ -7810,7 +7975,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>700</v>
       </c>
@@ -7830,7 +7995,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>702</v>
       </c>
@@ -7850,7 +8015,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>707</v>
       </c>
@@ -7870,7 +8035,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>708</v>
       </c>
@@ -7890,7 +8055,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>713</v>
       </c>
@@ -7910,7 +8075,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>45</v>
       </c>
@@ -7930,7 +8095,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>718</v>
       </c>
@@ -7950,7 +8115,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>720</v>
       </c>
@@ -7970,7 +8135,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>723</v>
       </c>
@@ -7990,7 +8155,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>728</v>
       </c>
@@ -8330,7 +8495,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>803</v>
       </c>
@@ -8350,7 +8515,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>805</v>
       </c>
@@ -8370,7 +8535,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>807</v>
       </c>
@@ -8390,7 +8555,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>812</v>
       </c>
@@ -8410,7 +8575,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>817</v>
       </c>
@@ -8430,7 +8595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>818</v>
       </c>
@@ -8450,7 +8615,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>821</v>
       </c>
@@ -8470,7 +8635,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>823</v>
       </c>
@@ -8490,7 +8655,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>828</v>
       </c>
@@ -8510,7 +8675,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>830</v>
       </c>
@@ -8530,7 +8695,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>831</v>
       </c>
@@ -8550,7 +8715,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>720</v>
       </c>
@@ -8570,7 +8735,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>836</v>
       </c>
@@ -8590,7 +8755,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>838</v>
       </c>
@@ -8610,7 +8775,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>843</v>
       </c>
@@ -8629,8 +8794,14 @@
       <c r="F207" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G207" s="2" t="s">
+        <v>1353</v>
+      </c>
+      <c r="H207" s="2" t="s">
+        <v>1354</v>
+      </c>
+    </row>
+    <row r="208" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>848</v>
       </c>
@@ -8650,7 +8821,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>79</v>
       </c>
@@ -8670,7 +8841,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>854</v>
       </c>
@@ -8690,7 +8861,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>859</v>
       </c>
@@ -8710,7 +8881,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>864</v>
       </c>
@@ -8729,8 +8900,14 @@
       <c r="F212" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G212" t="s">
+        <v>1361</v>
+      </c>
+      <c r="H212" s="2" t="s">
+        <v>1362</v>
+      </c>
+    </row>
+    <row r="213" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>869</v>
       </c>
@@ -8750,7 +8927,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>639</v>
       </c>
@@ -8770,7 +8947,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>874</v>
       </c>
@@ -8790,7 +8967,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>879</v>
       </c>
@@ -8810,7 +8987,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>884</v>
       </c>
@@ -8830,7 +9007,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>885</v>
       </c>
@@ -8850,7 +9027,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>888</v>
       </c>
@@ -8870,7 +9047,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>890</v>
       </c>
@@ -8890,7 +9067,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>895</v>
       </c>
@@ -8910,7 +9087,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>900</v>
       </c>
@@ -8930,7 +9107,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>644</v>
       </c>
@@ -8950,7 +9127,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>906</v>
       </c>
@@ -10570,7 +10747,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A305" t="s">
         <v>1202</v>
       </c>
@@ -10590,7 +10767,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A306" t="s">
         <v>1204</v>
       </c>
@@ -10610,7 +10787,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A307" t="s">
         <v>1209</v>
       </c>
@@ -10630,7 +10807,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="308" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A308" t="s">
         <v>1211</v>
       </c>
@@ -10650,7 +10827,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="309" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A309" t="s">
         <v>1216</v>
       </c>
@@ -10670,7 +10847,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="310" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A310" t="s">
         <v>1221</v>
       </c>
@@ -10690,7 +10867,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="311" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A311" t="s">
         <v>1226</v>
       </c>
@@ -10710,7 +10887,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="312" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A312" t="s">
         <v>1231</v>
       </c>
@@ -10730,7 +10907,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="313" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="313" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A313" t="s">
         <v>1236</v>
       </c>
@@ -10749,8 +10926,14 @@
       <c r="F313" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="314" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G313" s="2" t="s">
+        <v>1351</v>
+      </c>
+      <c r="H313" s="2" t="s">
+        <v>1352</v>
+      </c>
+    </row>
+    <row r="314" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A314" t="s">
         <v>1239</v>
       </c>
@@ -10770,7 +10953,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="315" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A315" t="s">
         <v>1244</v>
       </c>
@@ -10790,7 +10973,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="316" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A316" t="s">
         <v>1246</v>
       </c>
@@ -10810,7 +10993,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="317" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A317" t="s">
         <v>1251</v>
       </c>
@@ -10830,7 +11013,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="318" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A318" t="s">
         <v>1252</v>
       </c>
@@ -10850,7 +11033,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="319" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="319" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A319" t="s">
         <v>1257</v>
       </c>
@@ -10870,7 +11053,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="320" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A320" t="s">
         <v>1258</v>
       </c>
@@ -10890,7 +11073,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="321" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A321" t="s">
         <v>1263</v>
       </c>
@@ -10910,7 +11093,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="322" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A322" t="s">
         <v>1264</v>
       </c>
@@ -10930,7 +11113,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="323" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A323" t="s">
         <v>1269</v>
       </c>
@@ -10950,7 +11133,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="324" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="324" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A324" t="s">
         <v>1270</v>
       </c>
@@ -10969,8 +11152,14 @@
       <c r="F324" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="325" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G324" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="H324" s="2" t="s">
+        <v>1356</v>
+      </c>
+    </row>
+    <row r="325" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A325" t="s">
         <v>1275</v>
       </c>
@@ -10990,7 +11179,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="326" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A326" t="s">
         <v>1276</v>
       </c>
@@ -11010,7 +11199,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="327" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A327" t="s">
         <v>1278</v>
       </c>
@@ -11030,7 +11219,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="328" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A328" t="s">
         <v>1283</v>
       </c>
@@ -11050,7 +11239,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="329" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A329" t="s">
         <v>1288</v>
       </c>
@@ -11070,7 +11259,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="330" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A330" t="s">
         <v>1289</v>
       </c>
@@ -11090,7 +11279,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="331" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A331" t="s">
         <v>1294</v>
       </c>
@@ -11110,35 +11299,41 @@
         <v>11</v>
       </c>
     </row>
-    <row r="332" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A332" t="s">
+    <row r="332" spans="1:8" ht="302.39999999999998" x14ac:dyDescent="0.3">
+      <c r="A332" s="2" t="s">
+        <v>1363</v>
+      </c>
+      <c r="B332" t="s">
         <v>1299</v>
       </c>
-      <c r="B332" t="s">
+      <c r="C332" t="s">
         <v>1300</v>
       </c>
-      <c r="C332" t="s">
+      <c r="D332" t="s">
         <v>1301</v>
       </c>
-      <c r="D332" t="s">
+      <c r="E332" t="s">
         <v>1302</v>
-      </c>
-      <c r="E332" t="s">
-        <v>1303</v>
       </c>
       <c r="F332" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="333" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G332" t="s">
+        <v>1364</v>
+      </c>
+      <c r="H332" s="2" t="s">
+        <v>1365</v>
+      </c>
+    </row>
+    <row r="333" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A333" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B333" t="s">
         <v>1304</v>
       </c>
-      <c r="B333" t="s">
+      <c r="C333" t="s">
         <v>1305</v>
-      </c>
-      <c r="C333" t="s">
-        <v>1306</v>
       </c>
       <c r="D333" t="s">
         <v>721</v>
@@ -11150,61 +11345,61 @@
         <v>17</v>
       </c>
     </row>
-    <row r="334" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A334" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B334" t="s">
         <v>1307</v>
       </c>
-      <c r="B334" t="s">
+      <c r="C334" t="s">
         <v>1308</v>
       </c>
-      <c r="C334" t="s">
+      <c r="D334" t="s">
         <v>1309</v>
       </c>
-      <c r="D334" t="s">
+      <c r="E334" t="s">
         <v>1310</v>
-      </c>
-      <c r="E334" t="s">
-        <v>1311</v>
       </c>
       <c r="F334" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="335" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A335" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B335" t="s">
         <v>1312</v>
       </c>
-      <c r="B335" t="s">
+      <c r="C335" t="s">
         <v>1313</v>
       </c>
-      <c r="C335" t="s">
+      <c r="D335" t="s">
         <v>1314</v>
       </c>
-      <c r="D335" t="s">
+      <c r="E335" t="s">
         <v>1315</v>
       </c>
-      <c r="E335" t="s">
+      <c r="F335" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="336" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A336" t="s">
         <v>1316</v>
       </c>
-      <c r="F335" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="336" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A336" t="s">
+      <c r="B336" t="s">
         <v>1317</v>
       </c>
-      <c r="B336" t="s">
+      <c r="C336" t="s">
         <v>1318</v>
       </c>
-      <c r="C336" t="s">
+      <c r="D336" t="s">
         <v>1319</v>
       </c>
-      <c r="D336" t="s">
+      <c r="E336" t="s">
         <v>1320</v>
-      </c>
-      <c r="E336" t="s">
-        <v>1321</v>
       </c>
       <c r="F336" t="s">
         <v>17</v>
@@ -11212,19 +11407,19 @@
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A337" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B337" t="s">
         <v>1322</v>
       </c>
-      <c r="B337" t="s">
+      <c r="C337" t="s">
         <v>1323</v>
       </c>
-      <c r="C337" t="s">
+      <c r="D337" t="s">
         <v>1324</v>
       </c>
-      <c r="D337" t="s">
+      <c r="E337" t="s">
         <v>1325</v>
-      </c>
-      <c r="E337" t="s">
-        <v>1326</v>
       </c>
       <c r="F337" t="s">
         <v>17</v>
@@ -11232,16 +11427,16 @@
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A338" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B338" t="s">
         <v>1327</v>
-      </c>
-      <c r="B338" t="s">
-        <v>1328</v>
       </c>
       <c r="C338" t="s">
         <v>527</v>
       </c>
       <c r="D338" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="E338" t="s">
         <v>554</v>
@@ -11252,7 +11447,7 @@
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A339" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B339" t="s">
         <v>71</v>
@@ -11272,19 +11467,19 @@
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A340" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B340" t="s">
         <v>1331</v>
       </c>
-      <c r="B340" t="s">
+      <c r="C340" t="s">
         <v>1332</v>
       </c>
-      <c r="C340" t="s">
+      <c r="D340" t="s">
         <v>1333</v>
       </c>
-      <c r="D340" t="s">
+      <c r="E340" t="s">
         <v>1334</v>
-      </c>
-      <c r="E340" t="s">
-        <v>1335</v>
       </c>
       <c r="F340" t="s">
         <v>23</v>
@@ -11292,7 +11487,7 @@
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A341" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B341" t="s">
         <v>29</v>
@@ -11304,7 +11499,7 @@
         <v>360</v>
       </c>
       <c r="E341" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="F341" t="s">
         <v>42</v>
@@ -11312,19 +11507,19 @@
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A342" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B342" t="s">
         <v>1338</v>
       </c>
-      <c r="B342" t="s">
+      <c r="C342" t="s">
+        <v>1338</v>
+      </c>
+      <c r="D342" t="s">
         <v>1339</v>
       </c>
-      <c r="C342" t="s">
-        <v>1339</v>
-      </c>
-      <c r="D342" t="s">
+      <c r="E342" t="s">
         <v>1340</v>
-      </c>
-      <c r="E342" t="s">
-        <v>1341</v>
       </c>
       <c r="F342" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
docs: add partial answer's explaination
</commit_message>
<xml_diff>
--- a/raw_csv_quiz/Quiz_Week01.xlsx
+++ b/raw_csv_quiz/Quiz_Week01.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\LearningHub\ai-2y-journey\06-other\flashcard-app\raw_csv_quiz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6CF83C-71FA-4D32-98A3-14E9B0F82340}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C88BBAF0-5BF6-44E3-91CB-82DB5F054DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2076" uniqueCount="1366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2084" uniqueCount="1374">
   <si>
     <t>Question</t>
   </si>
@@ -4256,6 +4256,65 @@
   <si>
     <t>1. AWS is responsible for security OF the Cloud: Think Physical. AWS is responsible for the physical buildings, physical servers, physical network cables, the power, the cooling, and the hypervisor (the software that splits physical servers into virtual ones).
 2. The Customer is responsible for security IN the Cloud: Think Digital. You are responsible for everything you put inside the cloud. Your customer data, your passwords (IAM), your software, your application licenses, and your virtual firewall rules.</t>
+  </si>
+  <si>
+    <t>In the world of AWS, Availability Zones (AZs) are essentially distinct data centers (or groups of data centers) within a single Region. They are physically separated and have their own power, cooling, and networking.
+- The Single Point of Failure: If you provision your resources in only one Availability Zone (Option A), and that data center experiences a fire, flood, or massive power outage, your entire web application goes offline.
+- Redundancy: By using a minimum of two AZs, you ensure that if one goes down, the other is still running. AWS’s definition of "High Availability" starts at two because it creates a safety net where no single local disaster can take out your whole system.
+- Cost vs. Reliability: While you could use three or four AZs for even better "Fault Tolerance," the minimum requirement for a "Highly Available" architecture is two.</t>
+  </si>
+  <si>
+    <t>Think of Availability Zones like separate buildings on different sides of a city.
+- 1 AZ: You keep all your backup files in one building. If that building loses power, you're stuck.
+- 2 AZs: You keep a copy in Building A and a copy in Building B. Even if a lightning strike hits Building A, you can just drive to Building B and keep working.</t>
+  </si>
+  <si>
+    <t>B. Use a hybrid architecture that keeps tightly coupled local components in the private environment while extending compute and selected access services to the cloud.
+Why is this the answer?
+This question describes a classic "Real-World" scenario where a company can't just flip a switch and move everything to the cloud instantly. Here is the breakdown:
+"Approaching Capacity": This means they need more resources (Compute/Storage) fast. Expanding a physical data center (Option C) is slow and expensive.
+"Tightly Coupled" &amp; "Campus Network": The platform interacts with local systems on-site. Moving everything at once (Options A and D) would be a "Redesign" nightmare, which the company specifically wants to avoid.
+"Temporary Increases": This is known as Cloud Bursting. You keep your steady, everyday work in your own data center, but when you need extra power for a big study, you "burst" into the cloud to use its extra compute power temporarily.
+"External Collaborators": It is much easier and more secure to give external partners access to a specific "Slice" of data in the cloud (like an S3 bucket) than it is to let them into your private, on-campus network.</t>
+  </si>
+  <si>
+    <t>Imagine you have a small home kitchen (your private data center) that you use every day.
+The Problem: You are hosting a massive wedding (the genomics study) and need 10 extra ovens.
+Option B (Hybrid): You keep your home kitchen for your regular meals, but you rent a professional catering space (the Cloud) just for the wedding weekend. You have the extra space when you need it, and you don't have to tear down your house to build a giant kitchen you won't use next month.</t>
+  </si>
+  <si>
+    <t>C. Warm Standby.
+Why is this the answer?
+AWS defines Disaster Recovery (DR) strategies on a spectrum of cost vs. speed. This specific scenario describes a "scaled-down" version that is "fully functional."
+Fully Functional: This is the giveaway. In a Warm Standby, the secondary environment is already running. The databases are live, the application servers are on, and you can actually process a small amount of real traffic (like for testing) at any time.
+Reduced Capacity: To save money, you don't run the full fleet of servers. If your main region has 100 servers, your Warm Standby might only have 2.
+The Disaster Response: When the primary region fails, you simply use Auto Scaling to quickly "scale out" those 2 servers to 100. Because the "pilot" is already flying and the engines are warm, the switch is very fast.</t>
+  </si>
+  <si>
+    <t>Think of your Disaster Recovery plan like having a backup transportation plan:
+Backup and Restore: You have a box of car parts in your garage. If your main car breaks, you have to build a second car before you can drive. (Slowest)
+Pilot Light: You have a second car, but the battery is removed and the tires are flat. You need some time to get it ready. (Faster)
+Warm Standby: You have a small moped (scooter) in the garage. It’s running and ready to go right now, but it’s not as powerful as your car. If the car breaks, you take the moped and eventually upgrade it back to a car. (This Answer)
+Active/Active: You own two identical Ferraris and drive both of them simultaneously. (Fastest/Most Expensive)
+Key Exam Keyword: * "Core pieces/Database only" = Pilot Light.
+"Scaled-down/Fully functional" = Warm Standby.</t>
+  </si>
+  <si>
+    <t>To solve this, you have to look at the AWS hierarchy:
+Data Center: A single physical building with servers.
+Availability Zone (AZ): A group of one or more discrete data centers.
+Region: A geographic area that contains multiple, isolated Availability Zones.
+Multi-AZ (The Answer): This is specifically designed to protect you if one or more data centers (an entire AZ) fail. Because AZs are physically separated by miles but connected by low-latency fiber, if one "building" has a power outage, your app just runs in the other "building" in that same city (Region).
+Multi-Region: This protects you against a Region-wide disaster (like a massive hurricane hitting the entire East Coast or a major fiber cut affecting a whole state). While it does protect against data center failures, it is considered "overkill" for a single data center outage and is much more expensive and complex to set up.</t>
+  </si>
+  <si>
+    <t>Think of an AWS Region like New York City.
+Availability Zones are like different Boroughs (Manhattan, Brooklyn, Queens).
+Data Centers are the specific Buildings in those boroughs.
+If a transformer blows up in Manhattan (one data center/AZ fails), you can still run your business from your office in Brooklyn (another AZ). You are still "within the region" of New York City.
+You only move to Los Angeles (Multi-Region) if the entire East Coast is having a bad day.
+Key Exam Tip: * If the question says "Data Center failure" or "High Availability," think Multi-AZ.
+If the question says "Regional disaster," "Business Continuity," or "Global footprint," think Multi-Region.</t>
   </si>
 </sst>
 </file>
@@ -4951,7 +5010,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>79</v>
       </c>
@@ -4971,7 +5030,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -4991,7 +5050,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>89</v>
       </c>
@@ -5011,7 +5070,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>94</v>
       </c>
@@ -5031,7 +5090,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>99</v>
       </c>
@@ -5051,7 +5110,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>104</v>
       </c>
@@ -5071,7 +5130,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>109</v>
       </c>
@@ -5091,7 +5150,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>114</v>
       </c>
@@ -5111,7 +5170,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>119</v>
       </c>
@@ -5131,7 +5190,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>124</v>
       </c>
@@ -5151,7 +5210,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>129</v>
       </c>
@@ -5171,7 +5230,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>133</v>
       </c>
@@ -5191,7 +5250,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>138</v>
       </c>
@@ -5211,7 +5270,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>143</v>
       </c>
@@ -5230,8 +5289,14 @@
       <c r="F30" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G30" s="2" t="s">
+        <v>1370</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>1371</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>148</v>
       </c>
@@ -5251,7 +5316,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>153</v>
       </c>
@@ -5271,7 +5336,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>158</v>
       </c>
@@ -5291,7 +5356,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>159</v>
       </c>
@@ -5311,7 +5376,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>164</v>
       </c>
@@ -5331,7 +5396,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>169</v>
       </c>
@@ -5351,7 +5416,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>174</v>
       </c>
@@ -5371,7 +5436,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>179</v>
       </c>
@@ -5390,8 +5455,14 @@
       <c r="F38" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G38" s="2" t="s">
+        <v>1366</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>1367</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>184</v>
       </c>
@@ -5411,7 +5482,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>189</v>
       </c>
@@ -5431,7 +5502,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>194</v>
       </c>
@@ -5451,7 +5522,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>199</v>
       </c>
@@ -5471,7 +5542,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>204</v>
       </c>
@@ -5491,7 +5562,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>209</v>
       </c>
@@ -5511,7 +5582,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>214</v>
       </c>
@@ -5531,7 +5602,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>217</v>
       </c>
@@ -5551,7 +5622,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>222</v>
       </c>
@@ -5571,7 +5642,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>227</v>
       </c>
@@ -5911,7 +5982,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>304</v>
       </c>
@@ -5931,7 +6002,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>307</v>
       </c>
@@ -5950,8 +6021,14 @@
       <c r="F66" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G66" s="2" t="s">
+        <v>1372</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>1373</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>312</v>
       </c>
@@ -5971,7 +6048,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>316</v>
       </c>
@@ -5991,7 +6068,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>319</v>
       </c>
@@ -6011,7 +6088,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>322</v>
       </c>
@@ -6031,7 +6108,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>327</v>
       </c>
@@ -6051,7 +6128,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>329</v>
       </c>
@@ -6071,7 +6148,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>329</v>
       </c>
@@ -6091,7 +6168,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>338</v>
       </c>
@@ -6111,7 +6188,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>340</v>
       </c>
@@ -6131,7 +6208,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>343</v>
       </c>
@@ -6151,7 +6228,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>346</v>
       </c>
@@ -6171,7 +6248,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>347</v>
       </c>
@@ -6191,7 +6268,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>349</v>
       </c>
@@ -6211,7 +6288,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>352</v>
       </c>
@@ -7909,7 +7986,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="164" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>685</v>
       </c>
@@ -7927,6 +8004,12 @@
       </c>
       <c r="F164" t="s">
         <v>42</v>
+      </c>
+      <c r="G164" s="2" t="s">
+        <v>1368</v>
+      </c>
+      <c r="H164" s="2" t="s">
+        <v>1369</v>
       </c>
     </row>
     <row r="165" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">

</xml_diff>